<commit_message>
Read the FAA's winglet-equipped wingspan column
The workbook publishes wingspan in two columns —
`Wingspan_ft_without_winglets_sharklets` and
`Wingspan_ft_with_winglets_sharklets` — and the parser matched only the
first spelling it found. Types the FAA lists solely with winglets fitted
(`GLF6`, `E45X`, the E-Jets, …) therefore parsed with no wingspan at all,
which the builder rendered as 0 ft, and the second column was dropped for
every type that has one.

`ACDColumns` now tries header candidates in order, so the more specific
spelling claims its column before the broader one matches a neighbor, and
`Dimensions` carries `wingspanWithWinglets` alongside `wingspan`.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tests/SwiftACDTests/TestResources/sample_acd.xlsx
+++ b/Tests/SwiftACDTests/TestResources/sample_acd.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>ICAO Type Designator</t>
   </si>
@@ -31,7 +31,10 @@
     <t>MTOW (lbs)</t>
   </si>
   <si>
-    <t>Wingspan (ft)</t>
+    <t>Wingspan_ft_without_winglets_sharklets</t>
+  </si>
+  <si>
+    <t>Wingspan_ft_with_winglets_sharklets</t>
   </si>
   <si>
     <t>Length (ft)</t>
@@ -65,6 +68,9 @@
   </si>
   <si>
     <t>3</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>737-800W</t>
@@ -196,107 +202,116 @@
       <c r="M1" t="s">
         <v>12</v>
       </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G2">
         <v>174200</v>
       </c>
       <c r="H2">
-        <v>117.4</v>
-      </c>
-      <c r="I2">
+        <v>112.6</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2">
         <v>129.5</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>41.3</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>18.9</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>49.2</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>142</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
         <v>19</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" t="s">
-        <v>18</v>
       </c>
       <c r="G3">
         <v>174200</v>
       </c>
-      <c r="H3">
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3">
         <v>117.4</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>129.5</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>41.3</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>18.9</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>49.2</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>142</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G4">
         <v>169755</v>
@@ -305,39 +320,42 @@
         <v>111.8</v>
       </c>
       <c r="I4">
+        <v>117.5</v>
+      </c>
+      <c r="J4">
         <v>123.3</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>38.6</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>24.6</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>41.7</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>138</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G5">
         <v>2550</v>
@@ -345,40 +363,43 @@
       <c r="H5">
         <v>36.1</v>
       </c>
-      <c r="I5">
+      <c r="I5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5">
         <v>27.2</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>8.9</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>8.4</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <v>6.1</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>61</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G6">
         <v>987000</v>
@@ -386,40 +407,43 @@
       <c r="H6">
         <v>224.4</v>
       </c>
-      <c r="I6">
+      <c r="I6" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6">
         <v>250.2</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>63.5</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>36.1</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>116.8</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>154</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G7">
         <v>64500</v>
@@ -427,81 +451,87 @@
       <c r="H7">
         <v>93.3</v>
       </c>
-      <c r="I7">
+      <c r="I7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7">
         <v>107.8</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>27.4</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>24.6</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>38.0</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>121</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G8">
         <v>99600</v>
       </c>
-      <c r="H8">
+      <c r="H8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8">
         <v>99.6</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>99.7</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>25.6</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>14.8</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <v>39.1</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>132</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G9">
         <v>10000</v>
@@ -509,19 +539,22 @@
       <c r="H9">
         <v>40.0</v>
       </c>
-      <c r="I9">
+      <c r="I9" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9">
         <v>30.0</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>9.0</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>8.0</v>
       </c>
-      <c r="L9">
+      <c r="M9">
         <v>6.0</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill the wake category from the FAA where EUROCONTROL is silent
`Categories.wakeTurbulence` was sourced from EUROCONTROL alone, so the 143
profiles the APD does not list carried no wake category even though the FAA
publishes `ICAO_WTC` for every row of its workbook.

EUROCONTROL still wins where both publish one: it gives the ICAO letter,
while the FAA writes a coarser spelling. A type the FAA records as
straddling the 7,000 kg boundary (`"Light/Medium"`) is left empty rather
than rounded to one side — `AT8T` is the only type where that is the last
word, since EUROCONTROL categorizes the rest.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tests/SwiftACDTests/TestResources/sample_acd.xlsx
+++ b/Tests/SwiftACDTests/TestResources/sample_acd.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>ICAO Type Designator</t>
   </si>
@@ -28,6 +28,9 @@
     <t>TDG</t>
   </si>
   <si>
+    <t>ICAO_WTC</t>
+  </si>
+  <si>
     <t>MTOW (lbs)</t>
   </si>
   <si>
@@ -70,6 +73,9 @@
     <t>3</t>
   </si>
   <si>
+    <t>Medium</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -103,6 +109,9 @@
     <t>1A</t>
   </si>
   <si>
+    <t>Light</t>
+  </si>
+  <si>
     <t>B748</t>
   </si>
   <si>
@@ -118,6 +127,9 @@
     <t>7</t>
   </si>
   <si>
+    <t>Heavy</t>
+  </si>
+  <si>
     <t>DH8D</t>
   </si>
   <si>
@@ -128,6 +140,9 @@
   </si>
   <si>
     <t>B</t>
+  </si>
+  <si>
+    <t>Light/Medium</t>
   </si>
   <si>
     <t>GLF6</t>
@@ -205,356 +220,383 @@
       <c r="N1" t="s">
         <v>13</v>
       </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2">
+        <v>20</v>
+      </c>
+      <c r="G2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2">
         <v>174200</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>112.6</v>
       </c>
-      <c r="I2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2">
+      <c r="J2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2">
         <v>129.5</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>41.3</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>18.9</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>49.2</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>142</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
         <v>21</v>
       </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3">
+      <c r="H3">
         <v>174200</v>
       </c>
-      <c r="H3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3">
+      <c r="I3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3">
         <v>117.4</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>129.5</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>41.3</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>18.9</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>49.2</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>142</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4">
+        <v>20</v>
+      </c>
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4">
         <v>169755</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>111.8</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>117.5</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>123.3</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>38.6</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>24.6</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>41.7</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>138</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5">
+        <v>32</v>
+      </c>
+      <c r="G5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5">
         <v>2550</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>36.1</v>
       </c>
-      <c r="I5" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5">
+      <c r="J5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5">
         <v>27.2</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>8.9</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <v>8.4</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>6.1</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>61</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
-      </c>
-      <c r="G6">
+        <v>38</v>
+      </c>
+      <c r="G6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6">
         <v>987000</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>224.4</v>
       </c>
-      <c r="I6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6">
+      <c r="J6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6">
         <v>250.2</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>63.5</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>36.1</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>116.8</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>154</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7">
+        <v>20</v>
+      </c>
+      <c r="G7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7">
         <v>64500</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>93.3</v>
       </c>
-      <c r="I7" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7">
+      <c r="J7" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7">
         <v>107.8</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>27.4</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>24.6</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>38.0</v>
       </c>
-      <c r="N7">
+      <c r="O7">
         <v>121</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E8" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G8">
+        <v>49</v>
+      </c>
+      <c r="G8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8">
         <v>99600</v>
       </c>
-      <c r="H8" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8">
+      <c r="I8" t="s">
+        <v>22</v>
+      </c>
+      <c r="J8">
         <v>99.6</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>99.7</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>25.6</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <v>14.8</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>39.1</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>132</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9">
+        <v>20</v>
+      </c>
+      <c r="G9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H9">
         <v>10000</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>40.0</v>
       </c>
-      <c r="I9" t="s">
-        <v>20</v>
-      </c>
-      <c r="J9">
+      <c r="J9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K9">
         <v>30.0</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>9.0</v>
       </c>
-      <c r="L9">
+      <c r="M9">
         <v>8.0</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>6.0</v>
       </c>
-      <c r="N9">
+      <c r="O9">
         <v>100</v>
       </c>
     </row>

</xml_diff>